<commit_message>
Add LPI pillar re-fit, monthly scoring, and operational runbooks
- 00_fit_pillars.R: reproducible re-fit of both vulnerability pillars from
  phk_master.csv (all years); verified field-for-field vs the validated
  baseline (models_frozen_2025.rds). Enables annual re-calibration on new data.
- 07_freeze_calibration.R + 08_score_monthly.R: monthly LPI using frozen
  base-year weights/structure/scaling — only the pressure (LEI) input moves.
  Self-check reproduces the base-year annual LPI exactly.
- run_all.sh (annual full rebuild, now re-fits + promotes on verify) and
  run_monthly.sh (monthly update).
- README.md: LPI overview + annual/monthly runbooks + output/dashboard-handoff
  locations (lpi_scores.xlsx for records; lpi_data.js / lpi_monthly.js for the
  dashboard).
- Preserve immutable baseline models_frozen_2025.rds; gitignore regenerable
  intermediates.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/model_LPI/outputs/lpi_scores.xlsx
+++ b/model/model_LPI/outputs/lpi_scores.xlsx
@@ -7192,7 +7192,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.785</v>
+        <v>-0.785</v>
       </c>
       <c r="C2" t="n">
         <v>0.302</v>
@@ -7219,7 +7219,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.882</v>
+        <v>-0.882</v>
       </c>
       <c r="C3" t="n">
         <v>-0.08400000000000001</v>
@@ -7246,7 +7246,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.076</v>
+        <v>-0.076</v>
       </c>
       <c r="C4" t="n">
         <v>0.975</v>

</xml_diff>

<commit_message>
revising the LPI score calculation
</commit_message>
<xml_diff>
--- a/model/model_LPI/outputs/lpi_scores.xlsx
+++ b/model/model_LPI/outputs/lpi_scores.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>weighted sum of standardised pillars, min-max 0-100 within each year</t>
+          <t>weighted sum of the three 0-100 pillar scores (each normalised within its own index)</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:I139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -615,8 +615,7 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -652,20 +651,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>lpi_raw</t>
+          <t>lpi_rank</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>lpi_rank</t>
+          <t>tier</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>tier</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>tier_label</t>
         </is>
@@ -690,18 +684,15 @@
         <v>15.4</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>66.3</v>
       </c>
       <c r="G2" t="n">
-        <v>1.376</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -713,31 +704,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Papua Barat</t>
+          <t>Banten</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.4</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>44</v>
+        <v>68.8</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>30.5</v>
       </c>
       <c r="F3" t="n">
-        <v>90.8</v>
+        <v>59.5</v>
       </c>
       <c r="G3" t="n">
-        <v>1.119</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -749,31 +737,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Banten</t>
+          <t>Papua Barat</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>85.59999999999999</v>
+        <v>24.4</v>
       </c>
       <c r="D4" t="n">
-        <v>68.8</v>
+        <v>44</v>
       </c>
       <c r="E4" t="n">
-        <v>30.5</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>90.09999999999999</v>
+        <v>59.1</v>
       </c>
       <c r="G4" t="n">
-        <v>1.098</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" t="n">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -798,18 +783,15 @@
         <v>35.2</v>
       </c>
       <c r="F5" t="n">
-        <v>81.5</v>
+        <v>53.9</v>
       </c>
       <c r="G5" t="n">
-        <v>0.857</v>
+        <v>4</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I5" t="n">
         <v>1</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -834,18 +816,15 @@
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>80.90000000000001</v>
+        <v>52.5</v>
       </c>
       <c r="G6" t="n">
-        <v>0.839</v>
+        <v>5</v>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
-      </c>
-      <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -870,18 +849,15 @@
         <v>5.8</v>
       </c>
       <c r="F7" t="n">
-        <v>73.8</v>
+        <v>49.2</v>
       </c>
       <c r="G7" t="n">
-        <v>0.64</v>
+        <v>6</v>
       </c>
       <c r="H7" t="n">
-        <v>6</v>
-      </c>
-      <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -893,31 +869,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sulawesi Tengah</t>
+          <t>Maluku Utara</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>33.7</v>
+        <v>36.6</v>
       </c>
       <c r="D8" t="n">
-        <v>62.6</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="E8" t="n">
-        <v>43.6</v>
+        <v>20.4</v>
       </c>
       <c r="F8" t="n">
-        <v>70.2</v>
+        <v>46.9</v>
       </c>
       <c r="G8" t="n">
-        <v>0.539</v>
+        <v>7</v>
       </c>
       <c r="H8" t="n">
-        <v>7</v>
-      </c>
-      <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -929,31 +902,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Maluku Utara</t>
+          <t>Sulawesi Tengah</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>36.6</v>
+        <v>33.7</v>
       </c>
       <c r="D9" t="n">
-        <v>88.40000000000001</v>
+        <v>62.6</v>
       </c>
       <c r="E9" t="n">
-        <v>20.4</v>
+        <v>43.6</v>
       </c>
       <c r="F9" t="n">
-        <v>70</v>
+        <v>46.6</v>
       </c>
       <c r="G9" t="n">
-        <v>0.534</v>
+        <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>8</v>
-      </c>
-      <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -978,18 +948,15 @@
         <v>7.4</v>
       </c>
       <c r="F10" t="n">
-        <v>65</v>
+        <v>43.6</v>
       </c>
       <c r="G10" t="n">
-        <v>0.394</v>
+        <v>9</v>
       </c>
       <c r="H10" t="n">
-        <v>9</v>
-      </c>
-      <c r="I10" t="n">
         <v>2</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1014,18 +981,15 @@
         <v>19</v>
       </c>
       <c r="F11" t="n">
-        <v>58.8</v>
+        <v>39.3</v>
       </c>
       <c r="G11" t="n">
-        <v>0.219</v>
+        <v>10</v>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
-      </c>
-      <c r="I11" t="n">
         <v>2</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1050,18 +1014,15 @@
         <v>13.1</v>
       </c>
       <c r="F12" t="n">
-        <v>57.8</v>
+        <v>38.8</v>
       </c>
       <c r="G12" t="n">
-        <v>0.19</v>
+        <v>11</v>
       </c>
       <c r="H12" t="n">
-        <v>11</v>
-      </c>
-      <c r="I12" t="n">
         <v>2</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1073,31 +1034,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Jawa Timur</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>58.6</v>
+        <v>45</v>
       </c>
       <c r="D13" t="n">
-        <v>24.9</v>
+        <v>56.1</v>
       </c>
       <c r="E13" t="n">
-        <v>31.1</v>
+        <v>16.2</v>
       </c>
       <c r="F13" t="n">
-        <v>56.5</v>
+        <v>37.7</v>
       </c>
       <c r="G13" t="n">
-        <v>0.154</v>
+        <v>12</v>
       </c>
       <c r="H13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I13" t="n">
         <v>2</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1109,31 +1067,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jawa Timur</t>
+          <t>Bali</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>45</v>
+        <v>58.6</v>
       </c>
       <c r="D14" t="n">
-        <v>56.1</v>
+        <v>24.9</v>
       </c>
       <c r="E14" t="n">
-        <v>16.2</v>
+        <v>31.1</v>
       </c>
       <c r="F14" t="n">
-        <v>56</v>
+        <v>37.6</v>
       </c>
       <c r="G14" t="n">
-        <v>0.139</v>
+        <v>13</v>
       </c>
       <c r="H14" t="n">
-        <v>13</v>
-      </c>
-      <c r="I14" t="n">
         <v>2</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1158,18 +1113,15 @@
         <v>25.8</v>
       </c>
       <c r="F15" t="n">
-        <v>55.8</v>
+        <v>37.4</v>
       </c>
       <c r="G15" t="n">
-        <v>0.136</v>
+        <v>14</v>
       </c>
       <c r="H15" t="n">
-        <v>14</v>
-      </c>
-      <c r="I15" t="n">
         <v>2</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1181,31 +1133,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sulawesi Tenggara</t>
+          <t>Jawa Tengah</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>36.1</v>
+        <v>53.7</v>
       </c>
       <c r="D16" t="n">
-        <v>32.3</v>
+        <v>52.3</v>
       </c>
       <c r="E16" t="n">
-        <v>33.3</v>
+        <v>2.5</v>
       </c>
       <c r="F16" t="n">
-        <v>50.6</v>
+        <v>33.9</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.011</v>
+        <v>15</v>
       </c>
       <c r="H16" t="n">
-        <v>15</v>
-      </c>
-      <c r="I16" t="n">
         <v>2</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1217,31 +1166,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jawa Tengah</t>
+          <t>Sulawesi Tenggara</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>53.7</v>
+        <v>36.1</v>
       </c>
       <c r="D17" t="n">
-        <v>52.3</v>
+        <v>32.3</v>
       </c>
       <c r="E17" t="n">
-        <v>2.5</v>
+        <v>33.3</v>
       </c>
       <c r="F17" t="n">
-        <v>50</v>
+        <v>33.9</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.029</v>
+        <v>16</v>
       </c>
       <c r="H17" t="n">
-        <v>16</v>
-      </c>
-      <c r="I17" t="n">
         <v>2</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1266,18 +1212,15 @@
         <v>13.7</v>
       </c>
       <c r="F18" t="n">
-        <v>49.9</v>
+        <v>33.6</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.029</v>
+        <v>17</v>
       </c>
       <c r="H18" t="n">
-        <v>17</v>
-      </c>
-      <c r="I18" t="n">
         <v>2</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -1302,18 +1245,15 @@
         <v>17.9</v>
       </c>
       <c r="F19" t="n">
-        <v>48.5</v>
+        <v>32.6</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.07000000000000001</v>
+        <v>18</v>
       </c>
       <c r="H19" t="n">
-        <v>18</v>
-      </c>
-      <c r="I19" t="n">
         <v>3</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1338,18 +1278,15 @@
         <v>19.6</v>
       </c>
       <c r="F20" t="n">
-        <v>46.9</v>
+        <v>31.6</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.116</v>
+        <v>19</v>
       </c>
       <c r="H20" t="n">
-        <v>19</v>
-      </c>
-      <c r="I20" t="n">
         <v>3</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1374,18 +1311,15 @@
         <v>21.8</v>
       </c>
       <c r="F21" t="n">
-        <v>46.5</v>
+        <v>31.4</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.125</v>
+        <v>20</v>
       </c>
       <c r="H21" t="n">
-        <v>20</v>
-      </c>
-      <c r="I21" t="n">
         <v>3</v>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1410,18 +1344,15 @@
         <v>35</v>
       </c>
       <c r="F22" t="n">
-        <v>45.7</v>
+        <v>30.6</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.147</v>
+        <v>21</v>
       </c>
       <c r="H22" t="n">
-        <v>21</v>
-      </c>
-      <c r="I22" t="n">
         <v>3</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1446,18 +1377,15 @@
         <v>25</v>
       </c>
       <c r="F23" t="n">
-        <v>45.3</v>
+        <v>30.5</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.161</v>
+        <v>22</v>
       </c>
       <c r="H23" t="n">
-        <v>22</v>
-      </c>
-      <c r="I23" t="n">
         <v>3</v>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1469,31 +1397,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bengkulu</t>
+          <t>Kalimantan Selatan</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>29.8</v>
+        <v>38.9</v>
       </c>
       <c r="D24" t="n">
-        <v>24.1</v>
+        <v>50.4</v>
       </c>
       <c r="E24" t="n">
-        <v>34</v>
+        <v>4.9</v>
       </c>
       <c r="F24" t="n">
-        <v>44.1</v>
+        <v>29.7</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.194</v>
+        <v>23</v>
       </c>
       <c r="H24" t="n">
-        <v>23</v>
-      </c>
-      <c r="I24" t="n">
         <v>3</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1505,31 +1430,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kalimantan Selatan</t>
+          <t>Bengkulu</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>38.9</v>
+        <v>29.8</v>
       </c>
       <c r="D25" t="n">
-        <v>50.4</v>
+        <v>24.1</v>
       </c>
       <c r="E25" t="n">
-        <v>4.9</v>
+        <v>34</v>
       </c>
       <c r="F25" t="n">
-        <v>43.5</v>
+        <v>29.6</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.211</v>
+        <v>24</v>
       </c>
       <c r="H25" t="n">
-        <v>24</v>
-      </c>
-      <c r="I25" t="n">
         <v>3</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1554,18 +1476,15 @@
         <v>10.1</v>
       </c>
       <c r="F26" t="n">
-        <v>41.5</v>
+        <v>28.2</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.268</v>
+        <v>25</v>
       </c>
       <c r="H26" t="n">
-        <v>25</v>
-      </c>
-      <c r="I26" t="n">
         <v>3</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -1590,18 +1509,15 @@
         <v>25.3</v>
       </c>
       <c r="F27" t="n">
-        <v>40.4</v>
+        <v>27.3</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.297</v>
+        <v>26</v>
       </c>
       <c r="H27" t="n">
-        <v>26</v>
-      </c>
-      <c r="I27" t="n">
         <v>4</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1626,18 +1542,15 @@
         <v>19.5</v>
       </c>
       <c r="F28" t="n">
-        <v>37.4</v>
+        <v>25.5</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.381</v>
+        <v>27</v>
       </c>
       <c r="H28" t="n">
-        <v>27</v>
-      </c>
-      <c r="I28" t="n">
         <v>4</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1662,18 +1575,15 @@
         <v>13.5</v>
       </c>
       <c r="F29" t="n">
-        <v>36.8</v>
+        <v>25.2</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.399</v>
+        <v>28</v>
       </c>
       <c r="H29" t="n">
-        <v>28</v>
-      </c>
-      <c r="I29" t="n">
         <v>4</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1698,18 +1608,15 @@
         <v>33</v>
       </c>
       <c r="F30" t="n">
-        <v>32.9</v>
+        <v>22.3</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.509</v>
+        <v>29</v>
       </c>
       <c r="H30" t="n">
-        <v>29</v>
-      </c>
-      <c r="I30" t="n">
         <v>4</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1734,18 +1641,15 @@
         <v>19.6</v>
       </c>
       <c r="F31" t="n">
-        <v>30.4</v>
+        <v>20.8</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.578</v>
+        <v>30</v>
       </c>
       <c r="H31" t="n">
-        <v>30</v>
-      </c>
-      <c r="I31" t="n">
         <v>4</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1770,18 +1674,15 @@
         <v>13.5</v>
       </c>
       <c r="F32" t="n">
-        <v>18.4</v>
+        <v>13.2</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.915</v>
+        <v>31</v>
       </c>
       <c r="H32" t="n">
-        <v>31</v>
-      </c>
-      <c r="I32" t="n">
         <v>4</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1806,18 +1707,15 @@
         <v>2.8</v>
       </c>
       <c r="F33" t="n">
-        <v>14.1</v>
+        <v>10.7</v>
       </c>
       <c r="G33" t="n">
-        <v>-1.036</v>
+        <v>32</v>
       </c>
       <c r="H33" t="n">
-        <v>32</v>
-      </c>
-      <c r="I33" t="n">
         <v>4</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1842,18 +1740,15 @@
         <v>4.9</v>
       </c>
       <c r="F34" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="G34" t="n">
-        <v>-1.328</v>
+        <v>33</v>
       </c>
       <c r="H34" t="n">
-        <v>33</v>
-      </c>
-      <c r="I34" t="n">
         <v>4</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1878,18 +1773,15 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="G35" t="n">
-        <v>-1.432</v>
+        <v>34</v>
       </c>
       <c r="H35" t="n">
-        <v>34</v>
-      </c>
-      <c r="I35" t="n">
         <v>4</v>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -1914,18 +1806,15 @@
         <v>33.7</v>
       </c>
       <c r="F36" t="n">
-        <v>100</v>
+        <v>75.7</v>
       </c>
       <c r="G36" t="n">
-        <v>1.148</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
         <v>1</v>
       </c>
-      <c r="I36" t="n">
-        <v>1</v>
-      </c>
-      <c r="J36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -1950,18 +1839,15 @@
         <v>66.09999999999999</v>
       </c>
       <c r="F37" t="n">
-        <v>98.5</v>
+        <v>72.3</v>
       </c>
       <c r="G37" t="n">
-        <v>1.106</v>
+        <v>2</v>
       </c>
       <c r="H37" t="n">
-        <v>2</v>
-      </c>
-      <c r="I37" t="n">
         <v>1</v>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -1986,18 +1872,15 @@
         <v>68.2</v>
       </c>
       <c r="F38" t="n">
-        <v>96</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="G38" t="n">
-        <v>1.033</v>
+        <v>3</v>
       </c>
       <c r="H38" t="n">
-        <v>3</v>
-      </c>
-      <c r="I38" t="n">
         <v>1</v>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -2009,31 +1892,28 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Papua Barat</t>
+          <t>Kalimantan Timur</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>38.4</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="D39" t="n">
-        <v>43.6</v>
+        <v>49.5</v>
       </c>
       <c r="E39" t="n">
-        <v>92.3</v>
+        <v>60.3</v>
       </c>
       <c r="F39" t="n">
-        <v>81.2</v>
+        <v>60.9</v>
       </c>
       <c r="G39" t="n">
-        <v>0.607</v>
+        <v>4</v>
       </c>
       <c r="H39" t="n">
-        <v>4</v>
-      </c>
-      <c r="I39" t="n">
         <v>1</v>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -2045,31 +1925,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kalimantan Timur</t>
+          <t>Papua Barat</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>72.90000000000001</v>
+        <v>38.4</v>
       </c>
       <c r="D40" t="n">
-        <v>49.5</v>
+        <v>43.6</v>
       </c>
       <c r="E40" t="n">
-        <v>60.3</v>
+        <v>92.3</v>
       </c>
       <c r="F40" t="n">
-        <v>81.2</v>
+        <v>58.5</v>
       </c>
       <c r="G40" t="n">
-        <v>0.607</v>
+        <v>5</v>
       </c>
       <c r="H40" t="n">
-        <v>5</v>
-      </c>
-      <c r="I40" t="n">
         <v>1</v>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -2081,31 +1958,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>DI Yogyakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>45</v>
+        <v>60.2</v>
       </c>
       <c r="D41" t="n">
-        <v>26.2</v>
+        <v>57.3</v>
       </c>
       <c r="E41" t="n">
-        <v>100</v>
+        <v>57.7</v>
       </c>
       <c r="F41" t="n">
-        <v>80.7</v>
+        <v>58.4</v>
       </c>
       <c r="G41" t="n">
-        <v>0.593</v>
+        <v>6</v>
       </c>
       <c r="H41" t="n">
-        <v>6</v>
-      </c>
-      <c r="I41" t="n">
         <v>1</v>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -2117,31 +1991,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Kalimantan Selatan</t>
+          <t>DI Yogyakarta</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D42" t="n">
-        <v>42.7</v>
+        <v>26.2</v>
       </c>
       <c r="E42" t="n">
-        <v>89.5</v>
+        <v>100</v>
       </c>
       <c r="F42" t="n">
-        <v>79.3</v>
+        <v>57.6</v>
       </c>
       <c r="G42" t="n">
-        <v>0.552</v>
+        <v>7</v>
       </c>
       <c r="H42" t="n">
-        <v>7</v>
-      </c>
-      <c r="I42" t="n">
         <v>1</v>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -2153,31 +2024,28 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Jawa Barat</t>
+          <t>Kalimantan Selatan</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>60.2</v>
+        <v>39</v>
       </c>
       <c r="D43" t="n">
-        <v>57.3</v>
+        <v>42.7</v>
       </c>
       <c r="E43" t="n">
-        <v>57.7</v>
+        <v>89.5</v>
       </c>
       <c r="F43" t="n">
-        <v>77.2</v>
+        <v>57.4</v>
       </c>
       <c r="G43" t="n">
-        <v>0.493</v>
+        <v>8</v>
       </c>
       <c r="H43" t="n">
-        <v>8</v>
-      </c>
-      <c r="I43" t="n">
         <v>1</v>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -2202,18 +2070,15 @@
         <v>39.5</v>
       </c>
       <c r="F44" t="n">
-        <v>73.59999999999999</v>
+        <v>57.3</v>
       </c>
       <c r="G44" t="n">
-        <v>0.389</v>
+        <v>9</v>
       </c>
       <c r="H44" t="n">
-        <v>9</v>
-      </c>
-      <c r="I44" t="n">
         <v>2</v>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2238,18 +2103,15 @@
         <v>62.4</v>
       </c>
       <c r="F45" t="n">
-        <v>72.5</v>
+        <v>54.8</v>
       </c>
       <c r="G45" t="n">
-        <v>0.357</v>
+        <v>10</v>
       </c>
       <c r="H45" t="n">
-        <v>10</v>
-      </c>
-      <c r="I45" t="n">
         <v>2</v>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2274,18 +2136,15 @@
         <v>65.5</v>
       </c>
       <c r="F46" t="n">
-        <v>66.7</v>
+        <v>50.7</v>
       </c>
       <c r="G46" t="n">
-        <v>0.193</v>
+        <v>11</v>
       </c>
       <c r="H46" t="n">
-        <v>11</v>
-      </c>
-      <c r="I46" t="n">
         <v>2</v>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2297,31 +2156,28 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Jawa Timur</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>65.7</v>
+        <v>39.6</v>
       </c>
       <c r="D47" t="n">
-        <v>22.5</v>
+        <v>50.7</v>
       </c>
       <c r="E47" t="n">
-        <v>63.1</v>
+        <v>61.2</v>
       </c>
       <c r="F47" t="n">
-        <v>66.3</v>
+        <v>50.6</v>
       </c>
       <c r="G47" t="n">
-        <v>0.18</v>
+        <v>12</v>
       </c>
       <c r="H47" t="n">
-        <v>12</v>
-      </c>
-      <c r="I47" t="n">
         <v>2</v>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2333,31 +2189,28 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jawa Timur</t>
+          <t>Bali</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>39.6</v>
+        <v>65.7</v>
       </c>
       <c r="D48" t="n">
-        <v>50.7</v>
+        <v>22.5</v>
       </c>
       <c r="E48" t="n">
-        <v>61.2</v>
+        <v>63.1</v>
       </c>
       <c r="F48" t="n">
-        <v>66.2</v>
+        <v>50.6</v>
       </c>
       <c r="G48" t="n">
-        <v>0.176</v>
+        <v>13</v>
       </c>
       <c r="H48" t="n">
-        <v>13</v>
-      </c>
-      <c r="I48" t="n">
         <v>2</v>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2382,18 +2235,15 @@
         <v>61.2</v>
       </c>
       <c r="F49" t="n">
-        <v>63.8</v>
+        <v>49</v>
       </c>
       <c r="G49" t="n">
-        <v>0.108</v>
+        <v>14</v>
       </c>
       <c r="H49" t="n">
-        <v>14</v>
-      </c>
-      <c r="I49" t="n">
         <v>2</v>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2418,18 +2268,15 @@
         <v>76.7</v>
       </c>
       <c r="F50" t="n">
-        <v>63.4</v>
+        <v>47.6</v>
       </c>
       <c r="G50" t="n">
-        <v>0.096</v>
+        <v>15</v>
       </c>
       <c r="H50" t="n">
-        <v>15</v>
-      </c>
-      <c r="I50" t="n">
         <v>2</v>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2441,31 +2288,28 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Kalimantan Barat</t>
+          <t>Jawa Tengah</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>33</v>
+        <v>43.2</v>
       </c>
       <c r="D51" t="n">
-        <v>23.6</v>
+        <v>47.9</v>
       </c>
       <c r="E51" t="n">
-        <v>80.90000000000001</v>
+        <v>48.8</v>
       </c>
       <c r="F51" t="n">
-        <v>61.9</v>
+        <v>46.7</v>
       </c>
       <c r="G51" t="n">
-        <v>0.054</v>
+        <v>16</v>
       </c>
       <c r="H51" t="n">
-        <v>16</v>
-      </c>
-      <c r="I51" t="n">
         <v>2</v>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -2477,31 +2321,28 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Papua</t>
+          <t>Kalimantan Barat</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D52" t="n">
-        <v>13.1</v>
+        <v>23.6</v>
       </c>
       <c r="E52" t="n">
-        <v>92.3</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="F52" t="n">
-        <v>59.9</v>
+        <v>46.3</v>
       </c>
       <c r="G52" t="n">
-        <v>-0.004</v>
+        <v>17</v>
       </c>
       <c r="H52" t="n">
-        <v>17</v>
-      </c>
-      <c r="I52" t="n">
         <v>3</v>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2513,31 +2354,28 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jawa Tengah</t>
+          <t>Papua</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>43.2</v>
+        <v>25</v>
       </c>
       <c r="D53" t="n">
-        <v>47.9</v>
+        <v>13.1</v>
       </c>
       <c r="E53" t="n">
-        <v>48.8</v>
+        <v>92.3</v>
       </c>
       <c r="F53" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G53" t="n">
-        <v>-0.03</v>
+        <v>18</v>
       </c>
       <c r="H53" t="n">
-        <v>18</v>
-      </c>
-      <c r="I53" t="n">
         <v>3</v>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2562,18 +2400,15 @@
         <v>74.3</v>
       </c>
       <c r="F54" t="n">
-        <v>57.5</v>
+        <v>43.8</v>
       </c>
       <c r="G54" t="n">
-        <v>-0.07199999999999999</v>
+        <v>19</v>
       </c>
       <c r="H54" t="n">
-        <v>19</v>
-      </c>
-      <c r="I54" t="n">
         <v>3</v>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2585,31 +2420,28 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Sumatera Selatan</t>
+          <t>Sulawesi Utara</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>27.3</v>
+        <v>48.9</v>
       </c>
       <c r="D55" t="n">
-        <v>33.9</v>
+        <v>21.5</v>
       </c>
       <c r="E55" t="n">
-        <v>66.3</v>
+        <v>59</v>
       </c>
       <c r="F55" t="n">
-        <v>55.2</v>
+        <v>43.3</v>
       </c>
       <c r="G55" t="n">
-        <v>-0.139</v>
+        <v>20</v>
       </c>
       <c r="H55" t="n">
-        <v>20</v>
-      </c>
-      <c r="I55" t="n">
         <v>3</v>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2621,31 +2453,28 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Sulawesi Utara</t>
+          <t>Sumatera Selatan</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>48.9</v>
+        <v>27.3</v>
       </c>
       <c r="D56" t="n">
-        <v>21.5</v>
+        <v>33.9</v>
       </c>
       <c r="E56" t="n">
-        <v>59</v>
+        <v>66.3</v>
       </c>
       <c r="F56" t="n">
-        <v>55.2</v>
+        <v>42.8</v>
       </c>
       <c r="G56" t="n">
-        <v>-0.139</v>
+        <v>21</v>
       </c>
       <c r="H56" t="n">
-        <v>21</v>
-      </c>
-      <c r="I56" t="n">
         <v>3</v>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2670,18 +2499,15 @@
         <v>72.90000000000001</v>
       </c>
       <c r="F57" t="n">
-        <v>54.6</v>
+        <v>41.9</v>
       </c>
       <c r="G57" t="n">
-        <v>-0.155</v>
+        <v>22</v>
       </c>
       <c r="H57" t="n">
-        <v>22</v>
-      </c>
-      <c r="I57" t="n">
         <v>3</v>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2693,31 +2519,28 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Maluku</t>
+          <t>Riau</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>24</v>
+        <v>37.3</v>
       </c>
       <c r="D58" t="n">
-        <v>6.6</v>
+        <v>40</v>
       </c>
       <c r="E58" t="n">
-        <v>88.2</v>
+        <v>47.4</v>
       </c>
       <c r="F58" t="n">
-        <v>53.7</v>
+        <v>41.7</v>
       </c>
       <c r="G58" t="n">
-        <v>-0.18</v>
+        <v>23</v>
       </c>
       <c r="H58" t="n">
-        <v>23</v>
-      </c>
-      <c r="I58" t="n">
         <v>3</v>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2729,31 +2552,28 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Riau</t>
+          <t>Maluku</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>37.3</v>
+        <v>24</v>
       </c>
       <c r="D59" t="n">
-        <v>40</v>
+        <v>6.6</v>
       </c>
       <c r="E59" t="n">
-        <v>47.4</v>
+        <v>88.2</v>
       </c>
       <c r="F59" t="n">
-        <v>51.5</v>
+        <v>40.2</v>
       </c>
       <c r="G59" t="n">
-        <v>-0.246</v>
+        <v>24</v>
       </c>
       <c r="H59" t="n">
-        <v>24</v>
-      </c>
-      <c r="I59" t="n">
         <v>3</v>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -2778,18 +2598,15 @@
         <v>41.9</v>
       </c>
       <c r="F60" t="n">
-        <v>47.3</v>
+        <v>39.2</v>
       </c>
       <c r="G60" t="n">
-        <v>-0.366</v>
+        <v>25</v>
       </c>
       <c r="H60" t="n">
-        <v>25</v>
-      </c>
-      <c r="I60" t="n">
         <v>4</v>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -2814,18 +2631,15 @@
         <v>81.90000000000001</v>
       </c>
       <c r="F61" t="n">
-        <v>47.1</v>
+        <v>36.1</v>
       </c>
       <c r="G61" t="n">
-        <v>-0.37</v>
+        <v>26</v>
       </c>
       <c r="H61" t="n">
-        <v>26</v>
-      </c>
-      <c r="I61" t="n">
         <v>4</v>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -2850,18 +2664,15 @@
         <v>60.7</v>
       </c>
       <c r="F62" t="n">
-        <v>43.5</v>
+        <v>35.3</v>
       </c>
       <c r="G62" t="n">
-        <v>-0.473</v>
+        <v>27</v>
       </c>
       <c r="H62" t="n">
-        <v>27</v>
-      </c>
-      <c r="I62" t="n">
         <v>4</v>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="I62" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -2886,18 +2697,15 @@
         <v>59.3</v>
       </c>
       <c r="F63" t="n">
-        <v>42.5</v>
+        <v>34.7</v>
       </c>
       <c r="G63" t="n">
-        <v>-0.502</v>
+        <v>28</v>
       </c>
       <c r="H63" t="n">
-        <v>28</v>
-      </c>
-      <c r="I63" t="n">
         <v>4</v>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -2922,18 +2730,15 @@
         <v>63.3</v>
       </c>
       <c r="F64" t="n">
-        <v>42.4</v>
+        <v>34.3</v>
       </c>
       <c r="G64" t="n">
-        <v>-0.507</v>
+        <v>29</v>
       </c>
       <c r="H64" t="n">
-        <v>29</v>
-      </c>
-      <c r="I64" t="n">
         <v>4</v>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="I64" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -2958,18 +2763,15 @@
         <v>69.8</v>
       </c>
       <c r="F65" t="n">
-        <v>30.6</v>
+        <v>25.8</v>
       </c>
       <c r="G65" t="n">
-        <v>-0.844</v>
+        <v>30</v>
       </c>
       <c r="H65" t="n">
-        <v>30</v>
-      </c>
-      <c r="I65" t="n">
         <v>4</v>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -2994,18 +2796,15 @@
         <v>51.1</v>
       </c>
       <c r="F66" t="n">
-        <v>28.2</v>
+        <v>25.5</v>
       </c>
       <c r="G66" t="n">
-        <v>-0.915</v>
+        <v>31</v>
       </c>
       <c r="H66" t="n">
-        <v>31</v>
-      </c>
-      <c r="I66" t="n">
         <v>4</v>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -3030,18 +2829,15 @@
         <v>63.1</v>
       </c>
       <c r="F67" t="n">
-        <v>24.4</v>
+        <v>22.1</v>
       </c>
       <c r="G67" t="n">
-        <v>-1.024</v>
+        <v>32</v>
       </c>
       <c r="H67" t="n">
-        <v>32</v>
-      </c>
-      <c r="I67" t="n">
         <v>4</v>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="I67" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -3066,18 +2862,15 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
+        <v>10.2</v>
       </c>
       <c r="G68" t="n">
-        <v>-1.723</v>
+        <v>33</v>
       </c>
       <c r="H68" t="n">
-        <v>33</v>
-      </c>
-      <c r="I68" t="n">
         <v>4</v>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="I68" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -3102,18 +2895,15 @@
         <v>59</v>
       </c>
       <c r="F69" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="G69" t="n">
-        <v>1.78</v>
+        <v>1</v>
       </c>
       <c r="H69" t="n">
         <v>1</v>
       </c>
-      <c r="I69" t="n">
-        <v>1</v>
-      </c>
-      <c r="J69" t="inlineStr">
+      <c r="I69" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3138,18 +2928,15 @@
         <v>74.09999999999999</v>
       </c>
       <c r="F70" t="n">
-        <v>82.09999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="G70" t="n">
-        <v>1.227</v>
+        <v>2</v>
       </c>
       <c r="H70" t="n">
-        <v>2</v>
-      </c>
-      <c r="I70" t="n">
         <v>1</v>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="I70" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3174,18 +2961,15 @@
         <v>57.4</v>
       </c>
       <c r="F71" t="n">
-        <v>76.2</v>
+        <v>66.7</v>
       </c>
       <c r="G71" t="n">
-        <v>1.047</v>
+        <v>3</v>
       </c>
       <c r="H71" t="n">
-        <v>3</v>
-      </c>
-      <c r="I71" t="n">
         <v>1</v>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="I71" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3210,18 +2994,15 @@
         <v>59.9</v>
       </c>
       <c r="F72" t="n">
-        <v>64.5</v>
+        <v>59.1</v>
       </c>
       <c r="G72" t="n">
-        <v>0.6870000000000001</v>
+        <v>4</v>
       </c>
       <c r="H72" t="n">
-        <v>4</v>
-      </c>
-      <c r="I72" t="n">
         <v>1</v>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="I72" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3246,18 +3027,15 @@
         <v>95.59999999999999</v>
       </c>
       <c r="F73" t="n">
-        <v>61.7</v>
+        <v>57.8</v>
       </c>
       <c r="G73" t="n">
-        <v>0.6</v>
+        <v>5</v>
       </c>
       <c r="H73" t="n">
-        <v>5</v>
-      </c>
-      <c r="I73" t="n">
         <v>1</v>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3269,31 +3047,28 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Kalimantan Timur</t>
+          <t>Kalimantan Barat</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>71.40000000000001</v>
+        <v>34.9</v>
       </c>
       <c r="D74" t="n">
-        <v>47.1</v>
+        <v>24</v>
       </c>
       <c r="E74" t="n">
-        <v>52.2</v>
+        <v>100</v>
       </c>
       <c r="F74" t="n">
-        <v>61.4</v>
+        <v>56.8</v>
       </c>
       <c r="G74" t="n">
-        <v>0.59</v>
+        <v>6</v>
       </c>
       <c r="H74" t="n">
-        <v>6</v>
-      </c>
-      <c r="I74" t="n">
         <v>1</v>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3305,31 +3080,28 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Kalimantan Utara</t>
+          <t>Kalimantan Timur</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>54.4</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="D75" t="n">
-        <v>30.4</v>
+        <v>47.1</v>
       </c>
       <c r="E75" t="n">
-        <v>78.3</v>
+        <v>52.2</v>
       </c>
       <c r="F75" t="n">
-        <v>60.4</v>
+        <v>56.4</v>
       </c>
       <c r="G75" t="n">
-        <v>0.5600000000000001</v>
+        <v>7</v>
       </c>
       <c r="H75" t="n">
-        <v>7</v>
-      </c>
-      <c r="I75" t="n">
         <v>1</v>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="I75" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3341,31 +3113,28 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Kalimantan Barat</t>
+          <t>Sulawesi Tengah</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>34.9</v>
+        <v>35.3</v>
       </c>
       <c r="D76" t="n">
-        <v>24</v>
+        <v>78.5</v>
       </c>
       <c r="E76" t="n">
-        <v>100</v>
+        <v>55.3</v>
       </c>
       <c r="F76" t="n">
-        <v>60.2</v>
+        <v>56.4</v>
       </c>
       <c r="G76" t="n">
-        <v>0.555</v>
+        <v>8</v>
       </c>
       <c r="H76" t="n">
-        <v>8</v>
-      </c>
-      <c r="I76" t="n">
         <v>1</v>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="I76" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3377,31 +3146,28 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Sulawesi Tengah</t>
+          <t>Kalimantan Utara</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>35.3</v>
+        <v>54.4</v>
       </c>
       <c r="D77" t="n">
-        <v>78.5</v>
+        <v>30.4</v>
       </c>
       <c r="E77" t="n">
-        <v>55.3</v>
+        <v>78.3</v>
       </c>
       <c r="F77" t="n">
-        <v>59.7</v>
+        <v>56.3</v>
       </c>
       <c r="G77" t="n">
-        <v>0.54</v>
+        <v>9</v>
       </c>
       <c r="H77" t="n">
-        <v>9</v>
-      </c>
-      <c r="I77" t="n">
         <v>1</v>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="I77" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -3426,18 +3192,15 @@
         <v>27</v>
       </c>
       <c r="F78" t="n">
-        <v>56.8</v>
+        <v>53.9</v>
       </c>
       <c r="G78" t="n">
-        <v>0.45</v>
+        <v>10</v>
       </c>
       <c r="H78" t="n">
-        <v>10</v>
-      </c>
-      <c r="I78" t="n">
         <v>2</v>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="I78" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3462,18 +3225,15 @@
         <v>64.3</v>
       </c>
       <c r="F79" t="n">
-        <v>56.8</v>
+        <v>53.1</v>
       </c>
       <c r="G79" t="n">
-        <v>0.448</v>
+        <v>11</v>
       </c>
       <c r="H79" t="n">
-        <v>11</v>
-      </c>
-      <c r="I79" t="n">
         <v>2</v>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3498,18 +3258,15 @@
         <v>64.8</v>
       </c>
       <c r="F80" t="n">
-        <v>53.3</v>
+        <v>51.4</v>
       </c>
       <c r="G80" t="n">
-        <v>0.339</v>
+        <v>12</v>
       </c>
       <c r="H80" t="n">
-        <v>12</v>
-      </c>
-      <c r="I80" t="n">
         <v>2</v>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="I80" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3534,18 +3291,15 @@
         <v>65.09999999999999</v>
       </c>
       <c r="F81" t="n">
-        <v>52.1</v>
+        <v>50.1</v>
       </c>
       <c r="G81" t="n">
-        <v>0.305</v>
+        <v>13</v>
       </c>
       <c r="H81" t="n">
-        <v>13</v>
-      </c>
-      <c r="I81" t="n">
         <v>2</v>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="I81" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3570,18 +3324,15 @@
         <v>99</v>
       </c>
       <c r="F82" t="n">
-        <v>50.1</v>
+        <v>49.5</v>
       </c>
       <c r="G82" t="n">
-        <v>0.242</v>
+        <v>14</v>
       </c>
       <c r="H82" t="n">
-        <v>14</v>
-      </c>
-      <c r="I82" t="n">
         <v>2</v>
       </c>
-      <c r="J82" t="inlineStr">
+      <c r="I82" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3606,18 +3357,15 @@
         <v>43.8</v>
       </c>
       <c r="F83" t="n">
-        <v>47.5</v>
+        <v>46.9</v>
       </c>
       <c r="G83" t="n">
-        <v>0.163</v>
+        <v>15</v>
       </c>
       <c r="H83" t="n">
-        <v>15</v>
-      </c>
-      <c r="I83" t="n">
         <v>2</v>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="I83" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3642,18 +3390,15 @@
         <v>44.1</v>
       </c>
       <c r="F84" t="n">
-        <v>46.2</v>
+        <v>46.1</v>
       </c>
       <c r="G84" t="n">
-        <v>0.122</v>
+        <v>16</v>
       </c>
       <c r="H84" t="n">
-        <v>16</v>
-      </c>
-      <c r="I84" t="n">
         <v>2</v>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="I84" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3678,18 +3423,15 @@
         <v>70.90000000000001</v>
       </c>
       <c r="F85" t="n">
-        <v>45.8</v>
+        <v>46.1</v>
       </c>
       <c r="G85" t="n">
-        <v>0.11</v>
+        <v>17</v>
       </c>
       <c r="H85" t="n">
-        <v>17</v>
-      </c>
-      <c r="I85" t="n">
         <v>2</v>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="I85" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3717,15 +3459,12 @@
         <v>45.2</v>
       </c>
       <c r="G86" t="n">
-        <v>0.092</v>
+        <v>18</v>
       </c>
       <c r="H86" t="n">
-        <v>18</v>
-      </c>
-      <c r="I86" t="n">
         <v>2</v>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="I86" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -3750,18 +3489,15 @@
         <v>49.5</v>
       </c>
       <c r="F87" t="n">
-        <v>40.8</v>
+        <v>41.9</v>
       </c>
       <c r="G87" t="n">
-        <v>-0.043</v>
+        <v>19</v>
       </c>
       <c r="H87" t="n">
-        <v>19</v>
-      </c>
-      <c r="I87" t="n">
         <v>3</v>
       </c>
-      <c r="J87" t="inlineStr">
+      <c r="I87" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -3786,18 +3522,15 @@
         <v>43.6</v>
       </c>
       <c r="F88" t="n">
-        <v>39.5</v>
+        <v>41.3</v>
       </c>
       <c r="G88" t="n">
-        <v>-0.08400000000000001</v>
+        <v>20</v>
       </c>
       <c r="H88" t="n">
-        <v>20</v>
-      </c>
-      <c r="I88" t="n">
         <v>3</v>
       </c>
-      <c r="J88" t="inlineStr">
+      <c r="I88" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -3822,18 +3555,15 @@
         <v>80.09999999999999</v>
       </c>
       <c r="F89" t="n">
-        <v>37</v>
+        <v>40.4</v>
       </c>
       <c r="G89" t="n">
-        <v>-0.161</v>
+        <v>21</v>
       </c>
       <c r="H89" t="n">
-        <v>21</v>
-      </c>
-      <c r="I89" t="n">
         <v>3</v>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="I89" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -3858,18 +3588,15 @@
         <v>53.9</v>
       </c>
       <c r="F90" t="n">
-        <v>36.9</v>
+        <v>39.5</v>
       </c>
       <c r="G90" t="n">
-        <v>-0.164</v>
+        <v>22</v>
       </c>
       <c r="H90" t="n">
-        <v>22</v>
-      </c>
-      <c r="I90" t="n">
         <v>3</v>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="I90" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -3894,18 +3621,15 @@
         <v>53.3</v>
       </c>
       <c r="F91" t="n">
-        <v>33.9</v>
+        <v>37.3</v>
       </c>
       <c r="G91" t="n">
-        <v>-0.256</v>
+        <v>23</v>
       </c>
       <c r="H91" t="n">
-        <v>23</v>
-      </c>
-      <c r="I91" t="n">
         <v>3</v>
       </c>
-      <c r="J91" t="inlineStr">
+      <c r="I91" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -3930,18 +3654,15 @@
         <v>53.5</v>
       </c>
       <c r="F92" t="n">
-        <v>31</v>
+        <v>35.5</v>
       </c>
       <c r="G92" t="n">
-        <v>-0.347</v>
+        <v>24</v>
       </c>
       <c r="H92" t="n">
-        <v>24</v>
-      </c>
-      <c r="I92" t="n">
         <v>3</v>
       </c>
-      <c r="J92" t="inlineStr">
+      <c r="I92" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -3966,18 +3687,15 @@
         <v>40.5</v>
       </c>
       <c r="F93" t="n">
-        <v>30.5</v>
+        <v>35</v>
       </c>
       <c r="G93" t="n">
-        <v>-0.362</v>
+        <v>25</v>
       </c>
       <c r="H93" t="n">
-        <v>25</v>
-      </c>
-      <c r="I93" t="n">
         <v>3</v>
       </c>
-      <c r="J93" t="inlineStr">
+      <c r="I93" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -4002,18 +3720,15 @@
         <v>24.8</v>
       </c>
       <c r="F94" t="n">
-        <v>30.5</v>
+        <v>34.1</v>
       </c>
       <c r="G94" t="n">
-        <v>-0.363</v>
+        <v>26</v>
       </c>
       <c r="H94" t="n">
-        <v>26</v>
-      </c>
-      <c r="I94" t="n">
         <v>3</v>
       </c>
-      <c r="J94" t="inlineStr">
+      <c r="I94" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -4038,18 +3753,15 @@
         <v>48.7</v>
       </c>
       <c r="F95" t="n">
-        <v>29.2</v>
+        <v>34</v>
       </c>
       <c r="G95" t="n">
-        <v>-0.401</v>
+        <v>27</v>
       </c>
       <c r="H95" t="n">
-        <v>27</v>
-      </c>
-      <c r="I95" t="n">
         <v>3</v>
       </c>
-      <c r="J95" t="inlineStr">
+      <c r="I95" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -4074,18 +3786,15 @@
         <v>45.6</v>
       </c>
       <c r="F96" t="n">
-        <v>27.4</v>
+        <v>32.9</v>
       </c>
       <c r="G96" t="n">
-        <v>-0.458</v>
+        <v>28</v>
       </c>
       <c r="H96" t="n">
-        <v>28</v>
-      </c>
-      <c r="I96" t="n">
         <v>4</v>
       </c>
-      <c r="J96" t="inlineStr">
+      <c r="I96" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4110,18 +3819,15 @@
         <v>14.9</v>
       </c>
       <c r="F97" t="n">
-        <v>27.2</v>
+        <v>32.5</v>
       </c>
       <c r="G97" t="n">
-        <v>-0.464</v>
+        <v>29</v>
       </c>
       <c r="H97" t="n">
-        <v>29</v>
-      </c>
-      <c r="I97" t="n">
         <v>4</v>
       </c>
-      <c r="J97" t="inlineStr">
+      <c r="I97" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4146,18 +3852,15 @@
         <v>54.9</v>
       </c>
       <c r="F98" t="n">
-        <v>17</v>
+        <v>25.7</v>
       </c>
       <c r="G98" t="n">
-        <v>-0.777</v>
+        <v>30</v>
       </c>
       <c r="H98" t="n">
-        <v>30</v>
-      </c>
-      <c r="I98" t="n">
         <v>4</v>
       </c>
-      <c r="J98" t="inlineStr">
+      <c r="I98" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4182,18 +3885,15 @@
         <v>14.9</v>
       </c>
       <c r="F99" t="n">
-        <v>16.9</v>
+        <v>25</v>
       </c>
       <c r="G99" t="n">
-        <v>-0.78</v>
+        <v>31</v>
       </c>
       <c r="H99" t="n">
-        <v>31</v>
-      </c>
-      <c r="I99" t="n">
         <v>4</v>
       </c>
-      <c r="J99" t="inlineStr">
+      <c r="I99" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4218,18 +3918,15 @@
         <v>14.9</v>
       </c>
       <c r="F100" t="n">
-        <v>15.3</v>
+        <v>23.5</v>
       </c>
       <c r="G100" t="n">
-        <v>-0.831</v>
+        <v>32</v>
       </c>
       <c r="H100" t="n">
-        <v>32</v>
-      </c>
-      <c r="I100" t="n">
         <v>4</v>
       </c>
-      <c r="J100" t="inlineStr">
+      <c r="I100" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4254,18 +3951,15 @@
         <v>14.9</v>
       </c>
       <c r="F101" t="n">
-        <v>12.8</v>
+        <v>21.3</v>
       </c>
       <c r="G101" t="n">
-        <v>-0.907</v>
+        <v>33</v>
       </c>
       <c r="H101" t="n">
-        <v>33</v>
-      </c>
-      <c r="I101" t="n">
         <v>4</v>
       </c>
-      <c r="J101" t="inlineStr">
+      <c r="I101" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4290,18 +3984,15 @@
         <v>52.8</v>
       </c>
       <c r="F102" t="n">
-        <v>10</v>
+        <v>20.8</v>
       </c>
       <c r="G102" t="n">
-        <v>-0.993</v>
+        <v>34</v>
       </c>
       <c r="H102" t="n">
-        <v>34</v>
-      </c>
-      <c r="I102" t="n">
         <v>4</v>
       </c>
-      <c r="J102" t="inlineStr">
+      <c r="I102" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4326,18 +4017,15 @@
         <v>22.5</v>
       </c>
       <c r="F103" t="n">
-        <v>4.4</v>
+        <v>16.1</v>
       </c>
       <c r="G103" t="n">
-        <v>-1.165</v>
+        <v>35</v>
       </c>
       <c r="H103" t="n">
-        <v>35</v>
-      </c>
-      <c r="I103" t="n">
         <v>4</v>
       </c>
-      <c r="J103" t="inlineStr">
+      <c r="I103" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4362,18 +4050,15 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
-        <v>0</v>
+        <v>12.1</v>
       </c>
       <c r="G104" t="n">
-        <v>-1.302</v>
+        <v>36</v>
       </c>
       <c r="H104" t="n">
-        <v>36</v>
-      </c>
-      <c r="I104" t="n">
         <v>4</v>
       </c>
-      <c r="J104" t="inlineStr">
+      <c r="I104" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -4398,18 +4083,15 @@
         <v>76.40000000000001</v>
       </c>
       <c r="F105" t="n">
-        <v>100</v>
+        <v>88.7</v>
       </c>
       <c r="G105" t="n">
-        <v>1.924</v>
+        <v>1</v>
       </c>
       <c r="H105" t="n">
         <v>1</v>
       </c>
-      <c r="I105" t="n">
-        <v>1</v>
-      </c>
-      <c r="J105" t="inlineStr">
+      <c r="I105" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4434,18 +4116,15 @@
         <v>62.8</v>
       </c>
       <c r="F106" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="G106" t="n">
-        <v>0.882</v>
+        <v>2</v>
       </c>
       <c r="H106" t="n">
-        <v>2</v>
-      </c>
-      <c r="I106" t="n">
         <v>1</v>
       </c>
-      <c r="J106" t="inlineStr">
+      <c r="I106" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4457,31 +4136,28 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Kalimantan Utara</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>100</v>
+        <v>67.7</v>
       </c>
       <c r="D107" t="n">
-        <v>43.1</v>
+        <v>27</v>
       </c>
       <c r="E107" t="n">
-        <v>52.8</v>
+        <v>90.8</v>
       </c>
       <c r="F107" t="n">
-        <v>65.7</v>
+        <v>63.6</v>
       </c>
       <c r="G107" t="n">
-        <v>0.84</v>
+        <v>3</v>
       </c>
       <c r="H107" t="n">
-        <v>3</v>
-      </c>
-      <c r="I107" t="n">
         <v>1</v>
       </c>
-      <c r="J107" t="inlineStr">
+      <c r="I107" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4493,31 +4169,28 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Kalimantan Utara</t>
+          <t>DKI Jakarta</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>67.7</v>
+        <v>100</v>
       </c>
       <c r="D108" t="n">
-        <v>27</v>
+        <v>43.1</v>
       </c>
       <c r="E108" t="n">
-        <v>90.8</v>
+        <v>52.8</v>
       </c>
       <c r="F108" t="n">
-        <v>63.9</v>
+        <v>62</v>
       </c>
       <c r="G108" t="n">
-        <v>0.783</v>
+        <v>4</v>
       </c>
       <c r="H108" t="n">
-        <v>4</v>
-      </c>
-      <c r="I108" t="n">
         <v>1</v>
       </c>
-      <c r="J108" t="inlineStr">
+      <c r="I108" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4542,18 +4215,15 @@
         <v>64.8</v>
       </c>
       <c r="F109" t="n">
-        <v>59.7</v>
+        <v>59.2</v>
       </c>
       <c r="G109" t="n">
-        <v>0.652</v>
+        <v>5</v>
       </c>
       <c r="H109" t="n">
-        <v>5</v>
-      </c>
-      <c r="I109" t="n">
         <v>1</v>
       </c>
-      <c r="J109" t="inlineStr">
+      <c r="I109" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4565,31 +4235,28 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Maluku Utara</t>
+          <t>Sumatera Utara</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>45.7</v>
+        <v>45</v>
       </c>
       <c r="D110" t="n">
-        <v>100</v>
+        <v>26.6</v>
       </c>
       <c r="E110" t="n">
-        <v>24.7</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="F110" t="n">
-        <v>56.6</v>
+        <v>58.8</v>
       </c>
       <c r="G110" t="n">
-        <v>0.554</v>
+        <v>6</v>
       </c>
       <c r="H110" t="n">
-        <v>6</v>
-      </c>
-      <c r="I110" t="n">
         <v>1</v>
       </c>
-      <c r="J110" t="inlineStr">
+      <c r="I110" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4601,31 +4268,28 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Sumatera Utara</t>
+          <t>Sulawesi Selatan</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>45</v>
+        <v>41.8</v>
       </c>
       <c r="D111" t="n">
-        <v>26.6</v>
+        <v>21.6</v>
       </c>
       <c r="E111" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="F111" t="n">
-        <v>56.3</v>
+        <v>58.7</v>
       </c>
       <c r="G111" t="n">
-        <v>0.546</v>
+        <v>7</v>
       </c>
       <c r="H111" t="n">
-        <v>7</v>
-      </c>
-      <c r="I111" t="n">
         <v>1</v>
       </c>
-      <c r="J111" t="inlineStr">
+      <c r="I111" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4637,31 +4301,28 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Sulawesi Tengah</t>
+          <t>Kalimantan Barat</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>40.2</v>
+        <v>39.8</v>
       </c>
       <c r="D112" t="n">
-        <v>71.8</v>
+        <v>21.3</v>
       </c>
       <c r="E112" t="n">
-        <v>54.3</v>
+        <v>97.3</v>
       </c>
       <c r="F112" t="n">
-        <v>55.9</v>
+        <v>57</v>
       </c>
       <c r="G112" t="n">
-        <v>0.532</v>
+        <v>8</v>
       </c>
       <c r="H112" t="n">
-        <v>8</v>
-      </c>
-      <c r="I112" t="n">
         <v>1</v>
       </c>
-      <c r="J112" t="inlineStr">
+      <c r="I112" t="inlineStr">
         <is>
           <t>Risiko Sangat Tinggi</t>
         </is>
@@ -4673,31 +4334,28 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Sulawesi Selatan</t>
+          <t>Sulawesi Tengah</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>41.8</v>
+        <v>40.2</v>
       </c>
       <c r="D113" t="n">
-        <v>21.6</v>
+        <v>71.8</v>
       </c>
       <c r="E113" t="n">
-        <v>100</v>
+        <v>54.3</v>
       </c>
       <c r="F113" t="n">
-        <v>55.7</v>
+        <v>56.4</v>
       </c>
       <c r="G113" t="n">
-        <v>0.525</v>
+        <v>9</v>
       </c>
       <c r="H113" t="n">
-        <v>9</v>
-      </c>
-      <c r="I113" t="n">
         <v>2</v>
       </c>
-      <c r="J113" t="inlineStr">
+      <c r="I113" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4722,18 +4380,15 @@
         <v>78.2</v>
       </c>
       <c r="F114" t="n">
-        <v>54.1</v>
+        <v>56</v>
       </c>
       <c r="G114" t="n">
-        <v>0.476</v>
+        <v>10</v>
       </c>
       <c r="H114" t="n">
-        <v>10</v>
-      </c>
-      <c r="I114" t="n">
         <v>2</v>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="I114" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4745,31 +4400,28 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Kalimantan Timur</t>
+          <t>Maluku Utara</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>73.5</v>
+        <v>45.7</v>
       </c>
       <c r="D115" t="n">
-        <v>41.9</v>
+        <v>100</v>
       </c>
       <c r="E115" t="n">
-        <v>50.2</v>
+        <v>24.7</v>
       </c>
       <c r="F115" t="n">
-        <v>53.5</v>
+        <v>55.2</v>
       </c>
       <c r="G115" t="n">
-        <v>0.456</v>
+        <v>11</v>
       </c>
       <c r="H115" t="n">
-        <v>11</v>
-      </c>
-      <c r="I115" t="n">
         <v>2</v>
       </c>
-      <c r="J115" t="inlineStr">
+      <c r="I115" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4781,31 +4433,28 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Kalimantan Barat</t>
+          <t>Kalimantan Timur</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>39.8</v>
+        <v>73.5</v>
       </c>
       <c r="D116" t="n">
-        <v>21.3</v>
+        <v>41.9</v>
       </c>
       <c r="E116" t="n">
-        <v>97.3</v>
+        <v>50.2</v>
       </c>
       <c r="F116" t="n">
-        <v>53.5</v>
+        <v>53.6</v>
       </c>
       <c r="G116" t="n">
-        <v>0.456</v>
+        <v>12</v>
       </c>
       <c r="H116" t="n">
-        <v>12</v>
-      </c>
-      <c r="I116" t="n">
         <v>2</v>
       </c>
-      <c r="J116" t="inlineStr">
+      <c r="I116" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4830,18 +4479,15 @@
         <v>55.2</v>
       </c>
       <c r="F117" t="n">
-        <v>49</v>
+        <v>50.9</v>
       </c>
       <c r="G117" t="n">
-        <v>0.313</v>
+        <v>13</v>
       </c>
       <c r="H117" t="n">
-        <v>13</v>
-      </c>
-      <c r="I117" t="n">
         <v>2</v>
       </c>
-      <c r="J117" t="inlineStr">
+      <c r="I117" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4866,18 +4512,15 @@
         <v>59.7</v>
       </c>
       <c r="F118" t="n">
-        <v>48.7</v>
+        <v>50.5</v>
       </c>
       <c r="G118" t="n">
-        <v>0.304</v>
+        <v>14</v>
       </c>
       <c r="H118" t="n">
-        <v>14</v>
-      </c>
-      <c r="I118" t="n">
         <v>2</v>
       </c>
-      <c r="J118" t="inlineStr">
+      <c r="I118" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4902,18 +4545,15 @@
         <v>58.2</v>
       </c>
       <c r="F119" t="n">
-        <v>45</v>
+        <v>48.4</v>
       </c>
       <c r="G119" t="n">
-        <v>0.189</v>
+        <v>15</v>
       </c>
       <c r="H119" t="n">
-        <v>15</v>
-      </c>
-      <c r="I119" t="n">
         <v>2</v>
       </c>
-      <c r="J119" t="inlineStr">
+      <c r="I119" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4925,31 +4565,28 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Riau</t>
+          <t>Maluku</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>47.4</v>
+        <v>34.1</v>
       </c>
       <c r="D120" t="n">
-        <v>36.8</v>
+        <v>6.1</v>
       </c>
       <c r="E120" t="n">
-        <v>55.5</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="F120" t="n">
-        <v>43.5</v>
+        <v>48.1</v>
       </c>
       <c r="G120" t="n">
-        <v>0.142</v>
+        <v>16</v>
       </c>
       <c r="H120" t="n">
-        <v>16</v>
-      </c>
-      <c r="I120" t="n">
         <v>2</v>
       </c>
-      <c r="J120" t="inlineStr">
+      <c r="I120" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4961,31 +4598,28 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Jawa Timur</t>
+          <t>Riau</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>51.4</v>
+        <v>47.4</v>
       </c>
       <c r="D121" t="n">
-        <v>45.1</v>
+        <v>36.8</v>
       </c>
       <c r="E121" t="n">
-        <v>43.5</v>
+        <v>55.5</v>
       </c>
       <c r="F121" t="n">
-        <v>43.1</v>
+        <v>47.2</v>
       </c>
       <c r="G121" t="n">
-        <v>0.128</v>
+        <v>17</v>
       </c>
       <c r="H121" t="n">
-        <v>17</v>
-      </c>
-      <c r="I121" t="n">
         <v>2</v>
       </c>
-      <c r="J121" t="inlineStr">
+      <c r="I121" t="inlineStr">
         <is>
           <t>Risiko Tinggi</t>
         </is>
@@ -4997,31 +4631,28 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Maluku</t>
+          <t>Jawa Timur</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>34.1</v>
+        <v>51.4</v>
       </c>
       <c r="D122" t="n">
-        <v>6.1</v>
+        <v>45.1</v>
       </c>
       <c r="E122" t="n">
-        <v>91.59999999999999</v>
+        <v>43.5</v>
       </c>
       <c r="F122" t="n">
-        <v>41.7</v>
+        <v>46.1</v>
       </c>
       <c r="G122" t="n">
-        <v>0.08400000000000001</v>
+        <v>18</v>
       </c>
       <c r="H122" t="n">
-        <v>18</v>
-      </c>
-      <c r="I122" t="n">
         <v>3</v>
       </c>
-      <c r="J122" t="inlineStr">
+      <c r="I122" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5046,18 +4677,15 @@
         <v>52.8</v>
       </c>
       <c r="F123" t="n">
-        <v>40.9</v>
+        <v>44.7</v>
       </c>
       <c r="G123" t="n">
-        <v>0.058</v>
+        <v>19</v>
       </c>
       <c r="H123" t="n">
-        <v>19</v>
-      </c>
-      <c r="I123" t="n">
         <v>3</v>
       </c>
-      <c r="J123" t="inlineStr">
+      <c r="I123" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5082,18 +4710,15 @@
         <v>59.3</v>
       </c>
       <c r="F124" t="n">
-        <v>37.7</v>
+        <v>43.2</v>
       </c>
       <c r="G124" t="n">
-        <v>-0.044</v>
+        <v>20</v>
       </c>
       <c r="H124" t="n">
-        <v>20</v>
-      </c>
-      <c r="I124" t="n">
         <v>3</v>
       </c>
-      <c r="J124" t="inlineStr">
+      <c r="I124" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5118,18 +4743,15 @@
         <v>51.2</v>
       </c>
       <c r="F125" t="n">
-        <v>36.9</v>
+        <v>41.9</v>
       </c>
       <c r="G125" t="n">
-        <v>-0.067</v>
+        <v>21</v>
       </c>
       <c r="H125" t="n">
-        <v>21</v>
-      </c>
-      <c r="I125" t="n">
         <v>3</v>
       </c>
-      <c r="J125" t="inlineStr">
+      <c r="I125" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5141,31 +4763,28 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Sumatera Selatan</t>
+          <t>Nusa Tenggara Barat</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>36.2</v>
+        <v>21.8</v>
       </c>
       <c r="D126" t="n">
-        <v>29.7</v>
+        <v>15.3</v>
       </c>
       <c r="E126" t="n">
-        <v>48.2</v>
+        <v>71.8</v>
       </c>
       <c r="F126" t="n">
-        <v>32.5</v>
+        <v>39.9</v>
       </c>
       <c r="G126" t="n">
-        <v>-0.208</v>
+        <v>22</v>
       </c>
       <c r="H126" t="n">
-        <v>22</v>
-      </c>
-      <c r="I126" t="n">
         <v>3</v>
       </c>
-      <c r="J126" t="inlineStr">
+      <c r="I126" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5177,31 +4796,28 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Nusa Tenggara Barat</t>
+          <t>Sumatera Selatan</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>21.8</v>
+        <v>36.2</v>
       </c>
       <c r="D127" t="n">
-        <v>15.3</v>
+        <v>29.7</v>
       </c>
       <c r="E127" t="n">
-        <v>71.8</v>
+        <v>48.2</v>
       </c>
       <c r="F127" t="n">
-        <v>31.6</v>
+        <v>38.9</v>
       </c>
       <c r="G127" t="n">
-        <v>-0.236</v>
+        <v>23</v>
       </c>
       <c r="H127" t="n">
-        <v>23</v>
-      </c>
-      <c r="I127" t="n">
         <v>3</v>
       </c>
-      <c r="J127" t="inlineStr">
+      <c r="I127" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5226,18 +4842,15 @@
         <v>50.6</v>
       </c>
       <c r="F128" t="n">
-        <v>29.6</v>
+        <v>36.8</v>
       </c>
       <c r="G128" t="n">
-        <v>-0.299</v>
+        <v>24</v>
       </c>
       <c r="H128" t="n">
-        <v>24</v>
-      </c>
-      <c r="I128" t="n">
         <v>3</v>
       </c>
-      <c r="J128" t="inlineStr">
+      <c r="I128" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5262,18 +4875,15 @@
         <v>16.2</v>
       </c>
       <c r="F129" t="n">
-        <v>26</v>
+        <v>32.5</v>
       </c>
       <c r="G129" t="n">
-        <v>-0.412</v>
+        <v>25</v>
       </c>
       <c r="H129" t="n">
-        <v>25</v>
-      </c>
-      <c r="I129" t="n">
         <v>3</v>
       </c>
-      <c r="J129" t="inlineStr">
+      <c r="I129" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5298,18 +4908,15 @@
         <v>22.8</v>
       </c>
       <c r="F130" t="n">
-        <v>25.8</v>
+        <v>32.1</v>
       </c>
       <c r="G130" t="n">
-        <v>-0.417</v>
+        <v>26</v>
       </c>
       <c r="H130" t="n">
-        <v>26</v>
-      </c>
-      <c r="I130" t="n">
         <v>3</v>
       </c>
-      <c r="J130" t="inlineStr">
+      <c r="I130" t="inlineStr">
         <is>
           <t>Risiko Sedang</t>
         </is>
@@ -5321,31 +4928,28 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Papua Barat Daya</t>
+          <t>Sulawesi Barat</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>57.3</v>
+        <v>19.7</v>
       </c>
       <c r="D131" t="n">
-        <v>19.6</v>
+        <v>6.3</v>
       </c>
       <c r="E131" t="n">
-        <v>16.2</v>
+        <v>51.7</v>
       </c>
       <c r="F131" t="n">
-        <v>20.9</v>
+        <v>28.2</v>
       </c>
       <c r="G131" t="n">
-        <v>-0.571</v>
+        <v>27</v>
       </c>
       <c r="H131" t="n">
-        <v>27</v>
-      </c>
-      <c r="I131" t="n">
         <v>4</v>
       </c>
-      <c r="J131" t="inlineStr">
+      <c r="I131" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5357,31 +4961,28 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Sulawesi Barat</t>
+          <t>Papua Barat Daya</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>19.7</v>
+        <v>57.3</v>
       </c>
       <c r="D132" t="n">
-        <v>6.3</v>
+        <v>19.6</v>
       </c>
       <c r="E132" t="n">
-        <v>51.7</v>
+        <v>16.2</v>
       </c>
       <c r="F132" t="n">
-        <v>17.1</v>
+        <v>28.1</v>
       </c>
       <c r="G132" t="n">
-        <v>-0.6909999999999999</v>
+        <v>28</v>
       </c>
       <c r="H132" t="n">
-        <v>28</v>
-      </c>
-      <c r="I132" t="n">
         <v>4</v>
       </c>
-      <c r="J132" t="inlineStr">
+      <c r="I132" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5406,18 +5007,15 @@
         <v>50.3</v>
       </c>
       <c r="F133" t="n">
-        <v>14.1</v>
+        <v>25.9</v>
       </c>
       <c r="G133" t="n">
-        <v>-0.787</v>
+        <v>29</v>
       </c>
       <c r="H133" t="n">
-        <v>29</v>
-      </c>
-      <c r="I133" t="n">
         <v>4</v>
       </c>
-      <c r="J133" t="inlineStr">
+      <c r="I133" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5442,18 +5040,15 @@
         <v>18.2</v>
       </c>
       <c r="F134" t="n">
-        <v>11.7</v>
+        <v>22.2</v>
       </c>
       <c r="G134" t="n">
-        <v>-0.862</v>
+        <v>30</v>
       </c>
       <c r="H134" t="n">
-        <v>30</v>
-      </c>
-      <c r="I134" t="n">
         <v>4</v>
       </c>
-      <c r="J134" t="inlineStr">
+      <c r="I134" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5465,31 +5060,28 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Papua</t>
+          <t>Sumatera Barat</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>53.2</v>
+        <v>34</v>
       </c>
       <c r="D135" t="n">
-        <v>2.1</v>
+        <v>18.4</v>
       </c>
       <c r="E135" t="n">
-        <v>16.2</v>
+        <v>16.3</v>
       </c>
       <c r="F135" t="n">
-        <v>11.5</v>
+        <v>21.7</v>
       </c>
       <c r="G135" t="n">
-        <v>-0.87</v>
+        <v>31</v>
       </c>
       <c r="H135" t="n">
-        <v>31</v>
-      </c>
-      <c r="I135" t="n">
         <v>4</v>
       </c>
-      <c r="J135" t="inlineStr">
+      <c r="I135" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5501,31 +5093,28 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Sumatera Barat</t>
+          <t>Papua</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>34</v>
+        <v>53.2</v>
       </c>
       <c r="D136" t="n">
-        <v>18.4</v>
+        <v>2.1</v>
       </c>
       <c r="E136" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="F136" t="n">
-        <v>11.3</v>
+        <v>21.2</v>
       </c>
       <c r="G136" t="n">
-        <v>-0.874</v>
+        <v>32</v>
       </c>
       <c r="H136" t="n">
-        <v>32</v>
-      </c>
-      <c r="I136" t="n">
         <v>4</v>
       </c>
-      <c r="J136" t="inlineStr">
+      <c r="I136" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5550,18 +5139,15 @@
         <v>16.2</v>
       </c>
       <c r="F137" t="n">
-        <v>4.2</v>
+        <v>17.3</v>
       </c>
       <c r="G137" t="n">
-        <v>-1.101</v>
+        <v>33</v>
       </c>
       <c r="H137" t="n">
-        <v>33</v>
-      </c>
-      <c r="I137" t="n">
         <v>4</v>
       </c>
-      <c r="J137" t="inlineStr">
+      <c r="I137" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5573,31 +5159,28 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Gorontalo</t>
+          <t>Aceh</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>50.1</v>
+        <v>23.3</v>
       </c>
       <c r="D138" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
       <c r="E138" t="n">
-        <v>0</v>
+        <v>13.1</v>
       </c>
       <c r="F138" t="n">
-        <v>1.8</v>
+        <v>13.4</v>
       </c>
       <c r="G138" t="n">
-        <v>-1.174</v>
+        <v>34</v>
       </c>
       <c r="H138" t="n">
-        <v>34</v>
-      </c>
-      <c r="I138" t="n">
         <v>4</v>
       </c>
-      <c r="J138" t="inlineStr">
+      <c r="I138" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>
@@ -5609,31 +5192,28 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Aceh</t>
+          <t>Gorontalo</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>23.3</v>
+        <v>50.1</v>
       </c>
       <c r="D139" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
       <c r="E139" t="n">
-        <v>13.1</v>
+        <v>0</v>
       </c>
       <c r="F139" t="n">
-        <v>0</v>
+        <v>13.3</v>
       </c>
       <c r="G139" t="n">
-        <v>-1.232</v>
+        <v>35</v>
       </c>
       <c r="H139" t="n">
-        <v>35</v>
-      </c>
-      <c r="I139" t="n">
         <v>4</v>
       </c>
-      <c r="J139" t="inlineStr">
+      <c r="I139" t="inlineStr">
         <is>
           <t>Risiko Rendah</t>
         </is>

</xml_diff>

<commit_message>
Housekeeping: trim outputs/ to deliverable + inputs only
- Scripts 02/03/05/08 now write result tables ONLY into the workbook
  (via _xlsx_parts/) instead of redundant top-level CSVs, so the folder
  stays clean instead of byproducts reappearing each run.
- Removed stale orphans from the deleted 01 script (pillar_scores_*.csv,
  pillar_variable_spec.csv) and the now-unwritten CSVs.
- Untracked internal temp (_meta.csv, _lei_source.rds) and gitignored the
  transient report chart PNGs.
- outputs/ now tracks only: lpi_scores.xlsx (deliverable) + the 5 .rds inputs.
- Verified: full run + monthly run rebuild lpi_scores.xlsx (7 sheets incl.
  monthly); self-checks pass (diff 0).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/model_LPI/outputs/lpi_scores.xlsx
+++ b/model/model_LPI/outputs/lpi_scores.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>province-year</t>
+          <t>province-year (annual) + province-month (monthly sheet)</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Composite scaling</t>
+          <t>Aggregation</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>model_LEI/data/Komposit_LEI_Ketenagakerjaan.xlsx (LEI Per Provinsi, annual mean)</t>
+          <t>model_LEI/data/Komposit_LEI_Ketenagakerjaan.xlsx (LEI Per Provinsi)</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>model/model_LPI/code/ (01-06)</t>
+          <t>model/model_LPI/code/ (00-08)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename score columns to reflect true method (drop misleading _0_100)
The LPI is a weighted sum of the pillar scores, not a min-max 0-100
normalisation — and the MONTHLY LPI can exceed 0-100 when pressure moves
beyond the base-year range. So:
- columns renamed: pasar_kerja / struktural / tekanan / lpi (was *_0_100)
- workbook README sheet documents the columns + scale
- README/method text clarified: annual lands in 0-100, monthly can exceed

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/model_LPI/outputs/lpi_scores.xlsx
+++ b/model/model_LPI/outputs/lpi_scores.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -530,65 +530,89 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>weighted sum of the three 0-100 pillar scores (each normalised within its own index)</t>
+          <t>LPI = weighted sum of the three pillar scores (NOT re-normalised to 0-100)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PHK role</t>
+          <t>Columns</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>validation target only — never an input</t>
+          <t>pasar_kerja/struktural/tekanan = pillar index scores; lpi = their weighted sum; use `lpi`</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Source (labour+econ)</t>
+          <t>Scale</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>data/clean/phk_master.csv (via model_LPI pillar PCA)</t>
+          <t>pillars are min-max 0-100 in the base year; lpi is a weighted sum (annual lands in 0-100; MONTHLY values can exceed 0-100 when pressure moves beyond the base-year range)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Source (pressure)</t>
+          <t>PHK role</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>model_LEI/data/Komposit_LEI_Ketenagakerjaan.xlsx (LEI Per Provinsi)</t>
+          <t>validation target only — never an input</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Generated by</t>
+          <t>Source (labour+econ)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>model/model_LPI/code/ (00-08)</t>
+          <t>data/clean/phk_master.csv (via model_LPI pillar PCA)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Source (pressure)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>model_LEI/data/Komposit_LEI_Ketenagakerjaan.xlsx (LEI Per Provinsi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Generated by</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>model/model_LPI/code/ (00-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Build date</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -610,10 +634,10 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
@@ -632,22 +656,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>pasar_kerja_0_100</t>
+          <t>pasar_kerja</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>struktural_0_100</t>
+          <t>struktural</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>tekanan_0_100</t>
+          <t>tekanan</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>lpi_0_100</t>
+          <t>lpi</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -6864,10 +6888,10 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6888,22 +6912,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>lpi_0_100</t>
+          <t>lpi</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>pasar_kerja_0_100</t>
+          <t>pasar_kerja</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>struktural_0_100</t>
+          <t>struktural</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>tekanan_0_100</t>
+          <t>tekanan</t>
         </is>
       </c>
     </row>

</xml_diff>